<commit_message>
Updated Python code - Power and Temperature boundary
Updated Python code - Power and Temperature boundary
</commit_message>
<xml_diff>
--- a/code/ensemble_parameter_estimation/Python/Source_PowerDissipation_Temperature/Training_Data_1.xlsx
+++ b/code/ensemble_parameter_estimation/Python/Source_PowerDissipation_Temperature/Training_Data_1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trw1-my.sharepoint.com/personal/neel_padmanabhan_zf_com/Documents/Documents/EMB/AP/Thermal Analysis/ROM/Electronics_Motor_Disc/Rank 1 model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trw1-my.sharepoint.com/personal/neel_padmanabhan_zf_com/Documents/Documents/Paper/Github/Repository/Lumped-Parameter-Linear-Superposition-LPLSP/code/ensemble_parameter_estimation/Python/Source_PowerDissipation_Temperature/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="147" documentId="8_{366A8DC4-F71D-4209-BC64-C277DED7557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82917284-BCC2-4A9A-9883-EE991A2131A1}"/>
+  <xr:revisionPtr revIDLastSave="188" documentId="8_{366A8DC4-F71D-4209-BC64-C277DED7557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4313D40-8318-4F25-A842-AFA9E3694BCF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{951BE81E-92E2-42DD-8981-6F50081DAFB9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{951BE81E-92E2-42DD-8981-6F50081DAFB9}"/>
   </bookViews>
   <sheets>
     <sheet name="PowerDissipation_15s" sheetId="2" r:id="rId1"/>
@@ -40,174 +40,6 @@
     <t>t</t>
   </si>
   <si>
-    <t>P_Q2000</t>
-  </si>
-  <si>
-    <t>P_Q2001</t>
-  </si>
-  <si>
-    <t>P_Q2002</t>
-  </si>
-  <si>
-    <t>P_Q2003</t>
-  </si>
-  <si>
-    <t>P_Q2004</t>
-  </si>
-  <si>
-    <t>P_Q2005</t>
-  </si>
-  <si>
-    <t>P_R2016</t>
-  </si>
-  <si>
-    <t>P_L2000</t>
-  </si>
-  <si>
-    <t>P_Q1500</t>
-  </si>
-  <si>
-    <t>P_Q1501</t>
-  </si>
-  <si>
-    <t>P_Q11504</t>
-  </si>
-  <si>
-    <t>P_Q11505</t>
-  </si>
-  <si>
-    <t>P_C2012</t>
-  </si>
-  <si>
-    <t>P_C2013</t>
-  </si>
-  <si>
-    <t>P_C2077</t>
-  </si>
-  <si>
-    <t>P_IC20000</t>
-  </si>
-  <si>
-    <t>P_IC9000</t>
-  </si>
-  <si>
-    <t>P_IC10601</t>
-  </si>
-  <si>
-    <t>P_IC31900</t>
-  </si>
-  <si>
-    <t>T_Q2000_Junction</t>
-  </si>
-  <si>
-    <t>T_Q2000_Case</t>
-  </si>
-  <si>
-    <t>T_Q2001_Junction</t>
-  </si>
-  <si>
-    <t>T_Q2001_Case</t>
-  </si>
-  <si>
-    <t>T_Q2002_Junction</t>
-  </si>
-  <si>
-    <t>T_Q2002_Case</t>
-  </si>
-  <si>
-    <t>T_Q2003_Junction</t>
-  </si>
-  <si>
-    <t>T_Q2003_Case</t>
-  </si>
-  <si>
-    <t>T_Q2004_Junction</t>
-  </si>
-  <si>
-    <t>T_Q2004_Case</t>
-  </si>
-  <si>
-    <t>T_Q2005_Junction</t>
-  </si>
-  <si>
-    <t>T_Q2005_Case</t>
-  </si>
-  <si>
-    <t>T_R2016</t>
-  </si>
-  <si>
-    <t>T_L2000_Source</t>
-  </si>
-  <si>
-    <t>T_L2000_Case</t>
-  </si>
-  <si>
-    <t>T_Q1500_Junction</t>
-  </si>
-  <si>
-    <t>T_Q1500_Case</t>
-  </si>
-  <si>
-    <t>T_Q1501_Junction</t>
-  </si>
-  <si>
-    <t>T_Q1501_Case</t>
-  </si>
-  <si>
-    <t>T_Q11504_Junction</t>
-  </si>
-  <si>
-    <t>T_Q11504_Case</t>
-  </si>
-  <si>
-    <t>T_Q11505_Junction</t>
-  </si>
-  <si>
-    <t>T_Q11505_Case</t>
-  </si>
-  <si>
-    <t>T_C2012_Src</t>
-  </si>
-  <si>
-    <t>T_C2012_Case</t>
-  </si>
-  <si>
-    <t>T_C2013_Src</t>
-  </si>
-  <si>
-    <t>T_C2013_Case</t>
-  </si>
-  <si>
-    <t>T_C2077_Src</t>
-  </si>
-  <si>
-    <t>T_C2077_Case</t>
-  </si>
-  <si>
-    <t>T_IC20000_Src</t>
-  </si>
-  <si>
-    <t>T_IC20000_Case</t>
-  </si>
-  <si>
-    <t>T_IC9000_Src</t>
-  </si>
-  <si>
-    <t>T_IC9000_Case</t>
-  </si>
-  <si>
-    <t>T_IC10601_Src</t>
-  </si>
-  <si>
-    <t>T_IC10601_Case</t>
-  </si>
-  <si>
-    <t>T_IC31900</t>
-  </si>
-  <si>
-    <t>T_PCBA</t>
-  </si>
-  <si>
     <t>S_T1</t>
   </si>
   <si>
@@ -225,12 +57,180 @@
   <si>
     <t>T_S3</t>
   </si>
+  <si>
+    <t>P_1</t>
+  </si>
+  <si>
+    <t>P_2</t>
+  </si>
+  <si>
+    <t>P_3</t>
+  </si>
+  <si>
+    <t>P_4</t>
+  </si>
+  <si>
+    <t>P_5</t>
+  </si>
+  <si>
+    <t>P_6</t>
+  </si>
+  <si>
+    <t>P_7</t>
+  </si>
+  <si>
+    <t>P_8</t>
+  </si>
+  <si>
+    <t>P_9</t>
+  </si>
+  <si>
+    <t>P_10</t>
+  </si>
+  <si>
+    <t>P_11</t>
+  </si>
+  <si>
+    <t>P_12</t>
+  </si>
+  <si>
+    <t>P_13</t>
+  </si>
+  <si>
+    <t>P_14</t>
+  </si>
+  <si>
+    <t>P_15</t>
+  </si>
+  <si>
+    <t>P_16</t>
+  </si>
+  <si>
+    <t>P_17</t>
+  </si>
+  <si>
+    <t>P_18</t>
+  </si>
+  <si>
+    <t>P_19</t>
+  </si>
+  <si>
+    <t>T_1_Junction</t>
+  </si>
+  <si>
+    <t>T_1_Case</t>
+  </si>
+  <si>
+    <t>T_2_Junction</t>
+  </si>
+  <si>
+    <t>T_2_Case</t>
+  </si>
+  <si>
+    <t>T_3_Junction</t>
+  </si>
+  <si>
+    <t>T_3_Case</t>
+  </si>
+  <si>
+    <t>T_4_Junction</t>
+  </si>
+  <si>
+    <t>T_4_Case</t>
+  </si>
+  <si>
+    <t>T_5_Junction</t>
+  </si>
+  <si>
+    <t>T_5_Case</t>
+  </si>
+  <si>
+    <t>T_6_Junction</t>
+  </si>
+  <si>
+    <t>T_6_Case</t>
+  </si>
+  <si>
+    <t>T_7</t>
+  </si>
+  <si>
+    <t>T_8_Src</t>
+  </si>
+  <si>
+    <t>T_8_Case</t>
+  </si>
+  <si>
+    <t>T_9_Junction</t>
+  </si>
+  <si>
+    <t>T_9_Case</t>
+  </si>
+  <si>
+    <t>T_10_Junction</t>
+  </si>
+  <si>
+    <t>T_10_Case</t>
+  </si>
+  <si>
+    <t>T_11_Junction</t>
+  </si>
+  <si>
+    <t>T_11_Case</t>
+  </si>
+  <si>
+    <t>T_12_Junction</t>
+  </si>
+  <si>
+    <t>T_12_Case</t>
+  </si>
+  <si>
+    <t>T_13_Src</t>
+  </si>
+  <si>
+    <t>T_13_Case</t>
+  </si>
+  <si>
+    <t>T_14_Src</t>
+  </si>
+  <si>
+    <t>T_14_Case</t>
+  </si>
+  <si>
+    <t>T_15_Src</t>
+  </si>
+  <si>
+    <t>T_15_Case</t>
+  </si>
+  <si>
+    <t>T_16_Src</t>
+  </si>
+  <si>
+    <t>T_16_Case</t>
+  </si>
+  <si>
+    <t>T_17_Src</t>
+  </si>
+  <si>
+    <t>T_17_Case</t>
+  </si>
+  <si>
+    <t>T_18_Src</t>
+  </si>
+  <si>
+    <t>T_18_Case</t>
+  </si>
+  <si>
+    <t>T_19</t>
+  </si>
+  <si>
+    <t>T_PCB</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -254,6 +254,12 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Tahoma"/>
       <family val="2"/>
       <charset val="134"/>
@@ -316,10 +322,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -738,70 +740,70 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
@@ -3007,6 +3009,7 @@
     </row>
     <row r="39" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3032,70 +3035,70 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
@@ -4364,115 +4367,115 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="Z1" s="5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="AA1" s="5" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="AB1" s="5" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="AC1" s="5" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="AD1" s="5" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="AE1" s="5" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="AF1" s="5" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="AG1" s="5" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="AH1" s="5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="AI1" s="5" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="AJ1" s="5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="AK1" s="5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="AL1" s="5" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.2">

</xml_diff>